<commit_message>
Añadida carpeta y archivos
</commit_message>
<xml_diff>
--- a/Formato-archivos.xlsx
+++ b/Formato-archivos.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Usuario\Documents\Documentos Mari\Maestría en mecatrónica EU4M\Segundo Semestre\Proyecto mecatronico\Primer diseño preliminar\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Usuario\Documents\Documentos Mari\Maestría en mecatrónica EU4M\Segundo Semestre\Proyecto mecatronico\Diseño final\RoboticArmEU4M\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38CE1675-4C40-4C08-879E-AE533222B069}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A118839A-B607-4790-B5C4-9F07B16483BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20640" windowHeight="11040" activeTab="1" xr2:uid="{8A9B17CD-70AD-419F-A450-4EA25489036B}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="234" uniqueCount="120">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="235" uniqueCount="121">
   <si>
     <t>Ensamble</t>
   </si>
@@ -400,6 +400,9 @@
   </si>
   <si>
     <t>InsertoM4-2040617</t>
+  </si>
+  <si>
+    <t>Plano</t>
   </si>
 </sst>
 </file>
@@ -1081,7 +1084,7 @@
     <col min="2" max="2" width="17" customWidth="1"/>
     <col min="3" max="3" width="16.7109375" customWidth="1"/>
     <col min="4" max="4" width="32.85546875" customWidth="1"/>
-    <col min="5" max="5" width="9" customWidth="1"/>
+    <col min="5" max="5" width="24" customWidth="1"/>
     <col min="6" max="6" width="47.28515625" customWidth="1"/>
     <col min="8" max="8" width="26" customWidth="1"/>
     <col min="9" max="9" width="40.85546875" customWidth="1"/>
@@ -1113,6 +1116,9 @@
       <c r="D3" s="11" t="s">
         <v>25</v>
       </c>
+      <c r="E3" s="11" t="s">
+        <v>120</v>
+      </c>
       <c r="H3" s="3"/>
       <c r="I3" s="5"/>
     </row>

</xml_diff>